<commit_message>
feat: add prev abr-jun 2026 fix: consertar rótulos gráficos fix: consertar error label meses graficos
</commit_message>
<xml_diff>
--- a/data/accb_custo_total_itabuna.xlsx
+++ b/data/accb_custo_total_itabuna.xlsx
@@ -2628,7 +2628,14 @@
         <v>579.51999999999998</v>
       </c>
     </row>
-    <row r="256" ht="15.75" customHeight="1"/>
+    <row r="256" ht="15.75" customHeight="1">
+      <c r="A256" s="4">
+        <v>46082</v>
+      </c>
+      <c r="B256">
+        <v>612.80999999999995</v>
+      </c>
+    </row>
     <row r="257" ht="15.75" customHeight="1"/>
     <row r="258" ht="15.75" customHeight="1"/>
     <row r="259" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
feat: add prev mai-jul 2026
</commit_message>
<xml_diff>
--- a/data/accb_custo_total_itabuna.xlsx
+++ b/data/accb_custo_total_itabuna.xlsx
@@ -63,8 +63,11 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -584,11 +587,13 @@
   </sheetPr>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="6" width="14.42578125"/>
+    <col customWidth="1" min="1" max="1" width="14.42578125"/>
+    <col customWidth="1" min="2" max="2" style="1" width="14.42578125"/>
+    <col customWidth="1" min="3" max="6" width="14.42578125"/>
   </cols>
   <sheetData>
     <row r="1" ht="15.75" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -596,7 +601,7 @@
       </c>
     </row>
     <row r="2" ht="15.75" customHeight="1">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>38353</v>
       </c>
       <c r="B2" s="1">
@@ -604,7 +609,7 @@
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="2">
+      <c r="A3" s="3">
         <v>38384</v>
       </c>
       <c r="B3" s="1">
@@ -612,7 +617,7 @@
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="2">
+      <c r="A4" s="3">
         <v>38412</v>
       </c>
       <c r="B4" s="1">
@@ -620,7 +625,7 @@
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="2">
+      <c r="A5" s="3">
         <v>38443</v>
       </c>
       <c r="B5" s="1">
@@ -628,7 +633,7 @@
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="2">
+      <c r="A6" s="3">
         <v>38473</v>
       </c>
       <c r="B6" s="1">
@@ -636,7 +641,7 @@
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1">
-      <c r="A7" s="2">
+      <c r="A7" s="3">
         <v>38504</v>
       </c>
       <c r="B7" s="1">
@@ -644,7 +649,7 @@
       </c>
     </row>
     <row r="8" ht="15.75" customHeight="1">
-      <c r="A8" s="2">
+      <c r="A8" s="3">
         <v>38534</v>
       </c>
       <c r="B8" s="1">
@@ -652,7 +657,7 @@
       </c>
     </row>
     <row r="9" ht="15.75" customHeight="1">
-      <c r="A9" s="2">
+      <c r="A9" s="3">
         <v>38565</v>
       </c>
       <c r="B9" s="1">
@@ -660,7 +665,7 @@
       </c>
     </row>
     <row r="10" ht="15.75" customHeight="1">
-      <c r="A10" s="2">
+      <c r="A10" s="3">
         <v>38596</v>
       </c>
       <c r="B10" s="1">
@@ -668,7 +673,7 @@
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="2">
+      <c r="A11" s="3">
         <v>38626</v>
       </c>
       <c r="B11" s="1">
@@ -676,7 +681,7 @@
       </c>
     </row>
     <row r="12" ht="15.75" customHeight="1">
-      <c r="A12" s="2">
+      <c r="A12" s="3">
         <v>38657</v>
       </c>
       <c r="B12" s="1">
@@ -684,7 +689,7 @@
       </c>
     </row>
     <row r="13" ht="15.75" customHeight="1">
-      <c r="A13" s="2">
+      <c r="A13" s="3">
         <v>38687</v>
       </c>
       <c r="B13" s="1">
@@ -692,7 +697,7 @@
       </c>
     </row>
     <row r="14" ht="15.75" customHeight="1">
-      <c r="A14" s="2">
+      <c r="A14" s="3">
         <v>38718</v>
       </c>
       <c r="B14" s="1">
@@ -700,7 +705,7 @@
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1">
-      <c r="A15" s="2">
+      <c r="A15" s="3">
         <v>38749</v>
       </c>
       <c r="B15" s="1">
@@ -708,7 +713,7 @@
       </c>
     </row>
     <row r="16" ht="15.75" customHeight="1">
-      <c r="A16" s="2">
+      <c r="A16" s="3">
         <v>38777</v>
       </c>
       <c r="B16" s="1">
@@ -716,7 +721,7 @@
       </c>
     </row>
     <row r="17" ht="15.75" customHeight="1">
-      <c r="A17" s="2">
+      <c r="A17" s="3">
         <v>38808</v>
       </c>
       <c r="B17" s="1">
@@ -724,7 +729,7 @@
       </c>
     </row>
     <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="2">
+      <c r="A18" s="3">
         <v>38838</v>
       </c>
       <c r="B18" s="1">
@@ -732,7 +737,7 @@
       </c>
     </row>
     <row r="19" ht="15.75" customHeight="1">
-      <c r="A19" s="2">
+      <c r="A19" s="3">
         <v>38869</v>
       </c>
       <c r="B19" s="1">
@@ -740,7 +745,7 @@
       </c>
     </row>
     <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="2">
+      <c r="A20" s="3">
         <v>38899</v>
       </c>
       <c r="B20" s="1">
@@ -748,7 +753,7 @@
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="2">
+      <c r="A21" s="3">
         <v>38930</v>
       </c>
       <c r="B21" s="1">
@@ -756,7 +761,7 @@
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="2">
+      <c r="A22" s="3">
         <v>38961</v>
       </c>
       <c r="B22" s="1">
@@ -764,7 +769,7 @@
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="2">
+      <c r="A23" s="3">
         <v>38991</v>
       </c>
       <c r="B23" s="1">
@@ -772,7 +777,7 @@
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1">
-      <c r="A24" s="2">
+      <c r="A24" s="3">
         <v>39022</v>
       </c>
       <c r="B24" s="1">
@@ -780,7 +785,7 @@
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1">
-      <c r="A25" s="2">
+      <c r="A25" s="3">
         <v>39052</v>
       </c>
       <c r="B25" s="1">
@@ -788,7 +793,7 @@
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1">
-      <c r="A26" s="2">
+      <c r="A26" s="3">
         <v>39083</v>
       </c>
       <c r="B26" s="1">
@@ -796,7 +801,7 @@
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="2">
+      <c r="A27" s="3">
         <v>39114</v>
       </c>
       <c r="B27" s="1">
@@ -804,7 +809,7 @@
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1">
-      <c r="A28" s="2">
+      <c r="A28" s="3">
         <v>39142</v>
       </c>
       <c r="B28" s="1">
@@ -812,7 +817,7 @@
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1">
-      <c r="A29" s="2">
+      <c r="A29" s="3">
         <v>39173</v>
       </c>
       <c r="B29" s="1">
@@ -820,7 +825,7 @@
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="2">
+      <c r="A30" s="3">
         <v>39203</v>
       </c>
       <c r="B30" s="1">
@@ -828,7 +833,7 @@
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="2">
+      <c r="A31" s="3">
         <v>39234</v>
       </c>
       <c r="B31" s="1">
@@ -836,7 +841,7 @@
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="2">
+      <c r="A32" s="3">
         <v>39264</v>
       </c>
       <c r="B32" s="1">
@@ -844,7 +849,7 @@
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1">
-      <c r="A33" s="2">
+      <c r="A33" s="3">
         <v>39295</v>
       </c>
       <c r="B33" s="1">
@@ -852,7 +857,7 @@
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1">
-      <c r="A34" s="2">
+      <c r="A34" s="3">
         <v>39326</v>
       </c>
       <c r="B34" s="1">
@@ -860,7 +865,7 @@
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1">
-      <c r="A35" s="2">
+      <c r="A35" s="3">
         <v>39356</v>
       </c>
       <c r="B35" s="1">
@@ -868,7 +873,7 @@
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1">
-      <c r="A36" s="2">
+      <c r="A36" s="3">
         <v>39387</v>
       </c>
       <c r="B36" s="1">
@@ -876,7 +881,7 @@
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1">
-      <c r="A37" s="2">
+      <c r="A37" s="3">
         <v>39417</v>
       </c>
       <c r="B37" s="1">
@@ -884,7 +889,7 @@
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1">
-      <c r="A38" s="2">
+      <c r="A38" s="3">
         <v>39448</v>
       </c>
       <c r="B38" s="1">
@@ -892,7 +897,7 @@
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="A39" s="2">
+      <c r="A39" s="3">
         <v>39479</v>
       </c>
       <c r="B39" s="1">
@@ -900,7 +905,7 @@
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="A40" s="2">
+      <c r="A40" s="3">
         <v>39508</v>
       </c>
       <c r="B40" s="1">
@@ -908,7 +913,7 @@
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1">
-      <c r="A41" s="2">
+      <c r="A41" s="3">
         <v>39539</v>
       </c>
       <c r="B41" s="1">
@@ -916,7 +921,7 @@
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1">
-      <c r="A42" s="2">
+      <c r="A42" s="3">
         <v>39569</v>
       </c>
       <c r="B42" s="1">
@@ -924,7 +929,7 @@
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1">
-      <c r="A43" s="2">
+      <c r="A43" s="3">
         <v>39600</v>
       </c>
       <c r="B43" s="1">
@@ -932,7 +937,7 @@
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1">
-      <c r="A44" s="2">
+      <c r="A44" s="3">
         <v>39630</v>
       </c>
       <c r="B44" s="1">
@@ -940,7 +945,7 @@
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1">
-      <c r="A45" s="2">
+      <c r="A45" s="3">
         <v>39661</v>
       </c>
       <c r="B45" s="1">
@@ -948,7 +953,7 @@
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1">
-      <c r="A46" s="2">
+      <c r="A46" s="3">
         <v>39692</v>
       </c>
       <c r="B46" s="1">
@@ -956,7 +961,7 @@
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1">
-      <c r="A47" s="2">
+      <c r="A47" s="3">
         <v>39722</v>
       </c>
       <c r="B47" s="1">
@@ -964,7 +969,7 @@
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1">
-      <c r="A48" s="2">
+      <c r="A48" s="3">
         <v>39753</v>
       </c>
       <c r="B48" s="1">
@@ -972,7 +977,7 @@
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1">
-      <c r="A49" s="2">
+      <c r="A49" s="3">
         <v>39783</v>
       </c>
       <c r="B49" s="1">
@@ -980,7 +985,7 @@
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1">
-      <c r="A50" s="2">
+      <c r="A50" s="3">
         <v>39814</v>
       </c>
       <c r="B50" s="1">
@@ -988,7 +993,7 @@
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1">
-      <c r="A51" s="2">
+      <c r="A51" s="3">
         <v>39845</v>
       </c>
       <c r="B51" s="1">
@@ -996,7 +1001,7 @@
       </c>
     </row>
     <row r="52" ht="15.75" customHeight="1">
-      <c r="A52" s="2">
+      <c r="A52" s="3">
         <v>39873</v>
       </c>
       <c r="B52" s="1">
@@ -1004,7 +1009,7 @@
       </c>
     </row>
     <row r="53" ht="15.75" customHeight="1">
-      <c r="A53" s="2">
+      <c r="A53" s="3">
         <v>39904</v>
       </c>
       <c r="B53" s="1">
@@ -1012,7 +1017,7 @@
       </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
-      <c r="A54" s="2">
+      <c r="A54" s="3">
         <v>39934</v>
       </c>
       <c r="B54" s="1">
@@ -1020,7 +1025,7 @@
       </c>
     </row>
     <row r="55" ht="15.75" customHeight="1">
-      <c r="A55" s="2">
+      <c r="A55" s="3">
         <v>39965</v>
       </c>
       <c r="B55" s="1">
@@ -1028,7 +1033,7 @@
       </c>
     </row>
     <row r="56" ht="15.75" customHeight="1">
-      <c r="A56" s="2">
+      <c r="A56" s="3">
         <v>39995</v>
       </c>
       <c r="B56" s="1">
@@ -1036,7 +1041,7 @@
       </c>
     </row>
     <row r="57" ht="15.75" customHeight="1">
-      <c r="A57" s="2">
+      <c r="A57" s="3">
         <v>40026</v>
       </c>
       <c r="B57" s="1">
@@ -1044,7 +1049,7 @@
       </c>
     </row>
     <row r="58" ht="15.75" customHeight="1">
-      <c r="A58" s="2">
+      <c r="A58" s="3">
         <v>40057</v>
       </c>
       <c r="B58" s="1">
@@ -1052,7 +1057,7 @@
       </c>
     </row>
     <row r="59" ht="15.75" customHeight="1">
-      <c r="A59" s="2">
+      <c r="A59" s="3">
         <v>40087</v>
       </c>
       <c r="B59" s="1">
@@ -1060,7 +1065,7 @@
       </c>
     </row>
     <row r="60" ht="15.75" customHeight="1">
-      <c r="A60" s="2">
+      <c r="A60" s="3">
         <v>40118</v>
       </c>
       <c r="B60" s="1">
@@ -1068,7 +1073,7 @@
       </c>
     </row>
     <row r="61" ht="15.75" customHeight="1">
-      <c r="A61" s="2">
+      <c r="A61" s="3">
         <v>40148</v>
       </c>
       <c r="B61" s="1">
@@ -1076,7 +1081,7 @@
       </c>
     </row>
     <row r="62" ht="15.75" customHeight="1">
-      <c r="A62" s="2">
+      <c r="A62" s="3">
         <v>40179</v>
       </c>
       <c r="B62" s="1">
@@ -1084,7 +1089,7 @@
       </c>
     </row>
     <row r="63" ht="15.75" customHeight="1">
-      <c r="A63" s="2">
+      <c r="A63" s="3">
         <v>40210</v>
       </c>
       <c r="B63" s="1">
@@ -1092,7 +1097,7 @@
       </c>
     </row>
     <row r="64" ht="15.75" customHeight="1">
-      <c r="A64" s="2">
+      <c r="A64" s="3">
         <v>40238</v>
       </c>
       <c r="B64" s="1">
@@ -1100,7 +1105,7 @@
       </c>
     </row>
     <row r="65" ht="15.75" customHeight="1">
-      <c r="A65" s="2">
+      <c r="A65" s="3">
         <v>40269</v>
       </c>
       <c r="B65" s="1">
@@ -1108,7 +1113,7 @@
       </c>
     </row>
     <row r="66" ht="15.75" customHeight="1">
-      <c r="A66" s="2">
+      <c r="A66" s="3">
         <v>40299</v>
       </c>
       <c r="B66" s="1">
@@ -1116,7 +1121,7 @@
       </c>
     </row>
     <row r="67" ht="15.75" customHeight="1">
-      <c r="A67" s="2">
+      <c r="A67" s="3">
         <v>40330</v>
       </c>
       <c r="B67" s="1">
@@ -1124,7 +1129,7 @@
       </c>
     </row>
     <row r="68" ht="15.75" customHeight="1">
-      <c r="A68" s="2">
+      <c r="A68" s="3">
         <v>40360</v>
       </c>
       <c r="B68" s="1">
@@ -1132,7 +1137,7 @@
       </c>
     </row>
     <row r="69" ht="15.75" customHeight="1">
-      <c r="A69" s="2">
+      <c r="A69" s="3">
         <v>40391</v>
       </c>
       <c r="B69" s="1">
@@ -1140,7 +1145,7 @@
       </c>
     </row>
     <row r="70" ht="15.75" customHeight="1">
-      <c r="A70" s="2">
+      <c r="A70" s="3">
         <v>40422</v>
       </c>
       <c r="B70" s="1">
@@ -1148,7 +1153,7 @@
       </c>
     </row>
     <row r="71" ht="15.75" customHeight="1">
-      <c r="A71" s="2">
+      <c r="A71" s="3">
         <v>40452</v>
       </c>
       <c r="B71" s="1">
@@ -1156,7 +1161,7 @@
       </c>
     </row>
     <row r="72" ht="15.75" customHeight="1">
-      <c r="A72" s="2">
+      <c r="A72" s="3">
         <v>40483</v>
       </c>
       <c r="B72" s="1">
@@ -1164,7 +1169,7 @@
       </c>
     </row>
     <row r="73" ht="15.75" customHeight="1">
-      <c r="A73" s="2">
+      <c r="A73" s="3">
         <v>40513</v>
       </c>
       <c r="B73" s="1">
@@ -1172,7 +1177,7 @@
       </c>
     </row>
     <row r="74" ht="15.75" customHeight="1">
-      <c r="A74" s="2">
+      <c r="A74" s="3">
         <v>40544</v>
       </c>
       <c r="B74" s="1">
@@ -1180,7 +1185,7 @@
       </c>
     </row>
     <row r="75" ht="15.75" customHeight="1">
-      <c r="A75" s="2">
+      <c r="A75" s="3">
         <v>40575</v>
       </c>
       <c r="B75" s="1">
@@ -1188,7 +1193,7 @@
       </c>
     </row>
     <row r="76" ht="15.75" customHeight="1">
-      <c r="A76" s="2">
+      <c r="A76" s="3">
         <v>40603</v>
       </c>
       <c r="B76" s="1">
@@ -1196,7 +1201,7 @@
       </c>
     </row>
     <row r="77" ht="15.75" customHeight="1">
-      <c r="A77" s="2">
+      <c r="A77" s="3">
         <v>40634</v>
       </c>
       <c r="B77" s="1">
@@ -1204,7 +1209,7 @@
       </c>
     </row>
     <row r="78" ht="15.75" customHeight="1">
-      <c r="A78" s="2">
+      <c r="A78" s="3">
         <v>40664</v>
       </c>
       <c r="B78" s="1">
@@ -1212,7 +1217,7 @@
       </c>
     </row>
     <row r="79" ht="15.75" customHeight="1">
-      <c r="A79" s="2">
+      <c r="A79" s="3">
         <v>40695</v>
       </c>
       <c r="B79" s="1">
@@ -1220,7 +1225,7 @@
       </c>
     </row>
     <row r="80" ht="15.75" customHeight="1">
-      <c r="A80" s="2">
+      <c r="A80" s="3">
         <v>40725</v>
       </c>
       <c r="B80" s="1">
@@ -1228,7 +1233,7 @@
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1">
-      <c r="A81" s="2">
+      <c r="A81" s="3">
         <v>40756</v>
       </c>
       <c r="B81" s="1">
@@ -1236,7 +1241,7 @@
       </c>
     </row>
     <row r="82" ht="15.75" customHeight="1">
-      <c r="A82" s="2">
+      <c r="A82" s="3">
         <v>40787</v>
       </c>
       <c r="B82" s="1">
@@ -1244,7 +1249,7 @@
       </c>
     </row>
     <row r="83" ht="15.75" customHeight="1">
-      <c r="A83" s="2">
+      <c r="A83" s="3">
         <v>40817</v>
       </c>
       <c r="B83" s="1">
@@ -1252,7 +1257,7 @@
       </c>
     </row>
     <row r="84" ht="15.75" customHeight="1">
-      <c r="A84" s="2">
+      <c r="A84" s="3">
         <v>40848</v>
       </c>
       <c r="B84" s="1">
@@ -1260,7 +1265,7 @@
       </c>
     </row>
     <row r="85" ht="15.75" customHeight="1">
-      <c r="A85" s="2">
+      <c r="A85" s="3">
         <v>40878</v>
       </c>
       <c r="B85" s="1">
@@ -1268,7 +1273,7 @@
       </c>
     </row>
     <row r="86" ht="15.75" customHeight="1">
-      <c r="A86" s="2">
+      <c r="A86" s="3">
         <v>40909</v>
       </c>
       <c r="B86" s="1">
@@ -1276,7 +1281,7 @@
       </c>
     </row>
     <row r="87" ht="15.75" customHeight="1">
-      <c r="A87" s="2">
+      <c r="A87" s="3">
         <v>40940</v>
       </c>
       <c r="B87" s="1">
@@ -1284,7 +1289,7 @@
       </c>
     </row>
     <row r="88" ht="15.75" customHeight="1">
-      <c r="A88" s="2">
+      <c r="A88" s="3">
         <v>40969</v>
       </c>
       <c r="B88" s="1">
@@ -1292,7 +1297,7 @@
       </c>
     </row>
     <row r="89" ht="15.75" customHeight="1">
-      <c r="A89" s="2">
+      <c r="A89" s="3">
         <v>41000</v>
       </c>
       <c r="B89" s="1">
@@ -1300,7 +1305,7 @@
       </c>
     </row>
     <row r="90" ht="15.75" customHeight="1">
-      <c r="A90" s="2">
+      <c r="A90" s="3">
         <v>41030</v>
       </c>
       <c r="B90" s="1">
@@ -1308,7 +1313,7 @@
       </c>
     </row>
     <row r="91" ht="15.75" customHeight="1">
-      <c r="A91" s="2">
+      <c r="A91" s="3">
         <v>41061</v>
       </c>
       <c r="B91" s="1">
@@ -1316,7 +1321,7 @@
       </c>
     </row>
     <row r="92" ht="15.75" customHeight="1">
-      <c r="A92" s="2">
+      <c r="A92" s="3">
         <v>41091</v>
       </c>
       <c r="B92" s="1">
@@ -1324,7 +1329,7 @@
       </c>
     </row>
     <row r="93" ht="15.75" customHeight="1">
-      <c r="A93" s="2">
+      <c r="A93" s="3">
         <v>41122</v>
       </c>
       <c r="B93" s="1">
@@ -1332,7 +1337,7 @@
       </c>
     </row>
     <row r="94" ht="15.75" customHeight="1">
-      <c r="A94" s="2">
+      <c r="A94" s="3">
         <v>41153</v>
       </c>
       <c r="B94" s="1">
@@ -1340,7 +1345,7 @@
       </c>
     </row>
     <row r="95" ht="15.75" customHeight="1">
-      <c r="A95" s="2">
+      <c r="A95" s="3">
         <v>41183</v>
       </c>
       <c r="B95" s="1">
@@ -1348,7 +1353,7 @@
       </c>
     </row>
     <row r="96" ht="15.75" customHeight="1">
-      <c r="A96" s="2">
+      <c r="A96" s="3">
         <v>41214</v>
       </c>
       <c r="B96" s="1">
@@ -1356,7 +1361,7 @@
       </c>
     </row>
     <row r="97" ht="15.75" customHeight="1">
-      <c r="A97" s="2">
+      <c r="A97" s="3">
         <v>41244</v>
       </c>
       <c r="B97" s="1">
@@ -1364,7 +1369,7 @@
       </c>
     </row>
     <row r="98" ht="15.75" customHeight="1">
-      <c r="A98" s="2">
+      <c r="A98" s="3">
         <v>41275</v>
       </c>
       <c r="B98" s="1">
@@ -1372,7 +1377,7 @@
       </c>
     </row>
     <row r="99" ht="15.75" customHeight="1">
-      <c r="A99" s="2">
+      <c r="A99" s="3">
         <v>41306</v>
       </c>
       <c r="B99" s="1">
@@ -1380,7 +1385,7 @@
       </c>
     </row>
     <row r="100" ht="15.75" customHeight="1">
-      <c r="A100" s="2">
+      <c r="A100" s="3">
         <v>41334</v>
       </c>
       <c r="B100" s="1">
@@ -1388,7 +1393,7 @@
       </c>
     </row>
     <row r="101" ht="15.75" customHeight="1">
-      <c r="A101" s="2">
+      <c r="A101" s="3">
         <v>41365</v>
       </c>
       <c r="B101" s="1">
@@ -1396,7 +1401,7 @@
       </c>
     </row>
     <row r="102" ht="15.75" customHeight="1">
-      <c r="A102" s="2">
+      <c r="A102" s="3">
         <v>41395</v>
       </c>
       <c r="B102" s="1">
@@ -1404,7 +1409,7 @@
       </c>
     </row>
     <row r="103" ht="15.75" customHeight="1">
-      <c r="A103" s="2">
+      <c r="A103" s="3">
         <v>41426</v>
       </c>
       <c r="B103" s="1">
@@ -1412,7 +1417,7 @@
       </c>
     </row>
     <row r="104" ht="15.75" customHeight="1">
-      <c r="A104" s="2">
+      <c r="A104" s="3">
         <v>41456</v>
       </c>
       <c r="B104" s="1">
@@ -1420,7 +1425,7 @@
       </c>
     </row>
     <row r="105" ht="15.75" customHeight="1">
-      <c r="A105" s="2">
+      <c r="A105" s="3">
         <v>41487</v>
       </c>
       <c r="B105" s="1">
@@ -1428,7 +1433,7 @@
       </c>
     </row>
     <row r="106" ht="15.75" customHeight="1">
-      <c r="A106" s="2">
+      <c r="A106" s="3">
         <v>41518</v>
       </c>
       <c r="B106" s="1">
@@ -1436,7 +1441,7 @@
       </c>
     </row>
     <row r="107" ht="15.75" customHeight="1">
-      <c r="A107" s="2">
+      <c r="A107" s="3">
         <v>41548</v>
       </c>
       <c r="B107" s="1">
@@ -1444,7 +1449,7 @@
       </c>
     </row>
     <row r="108" ht="15.75" customHeight="1">
-      <c r="A108" s="2">
+      <c r="A108" s="3">
         <v>41579</v>
       </c>
       <c r="B108" s="1">
@@ -1452,7 +1457,7 @@
       </c>
     </row>
     <row r="109" ht="15.75" customHeight="1">
-      <c r="A109" s="2">
+      <c r="A109" s="3">
         <v>41609</v>
       </c>
       <c r="B109" s="1">
@@ -1460,7 +1465,7 @@
       </c>
     </row>
     <row r="110" ht="15.75" customHeight="1">
-      <c r="A110" s="2">
+      <c r="A110" s="3">
         <v>41640</v>
       </c>
       <c r="B110" s="1">
@@ -1468,7 +1473,7 @@
       </c>
     </row>
     <row r="111" ht="15.75" customHeight="1">
-      <c r="A111" s="2">
+      <c r="A111" s="3">
         <v>41671</v>
       </c>
       <c r="B111" s="1">
@@ -1476,7 +1481,7 @@
       </c>
     </row>
     <row r="112" ht="15.75" customHeight="1">
-      <c r="A112" s="2">
+      <c r="A112" s="3">
         <v>41699</v>
       </c>
       <c r="B112" s="1">
@@ -1484,7 +1489,7 @@
       </c>
     </row>
     <row r="113" ht="15.75" customHeight="1">
-      <c r="A113" s="2">
+      <c r="A113" s="3">
         <v>41730</v>
       </c>
       <c r="B113" s="1">
@@ -1492,7 +1497,7 @@
       </c>
     </row>
     <row r="114" ht="15.75" customHeight="1">
-      <c r="A114" s="2">
+      <c r="A114" s="3">
         <v>41760</v>
       </c>
       <c r="B114" s="1">
@@ -1500,7 +1505,7 @@
       </c>
     </row>
     <row r="115" ht="15.75" customHeight="1">
-      <c r="A115" s="2">
+      <c r="A115" s="3">
         <v>41791</v>
       </c>
       <c r="B115" s="1">
@@ -1508,7 +1513,7 @@
       </c>
     </row>
     <row r="116" ht="15.75" customHeight="1">
-      <c r="A116" s="2">
+      <c r="A116" s="3">
         <v>41821</v>
       </c>
       <c r="B116" s="1">
@@ -1516,7 +1521,7 @@
       </c>
     </row>
     <row r="117" ht="15.75" customHeight="1">
-      <c r="A117" s="2">
+      <c r="A117" s="3">
         <v>41852</v>
       </c>
       <c r="B117" s="1">
@@ -1524,7 +1529,7 @@
       </c>
     </row>
     <row r="118" ht="15.75" customHeight="1">
-      <c r="A118" s="2">
+      <c r="A118" s="3">
         <v>41883</v>
       </c>
       <c r="B118" s="1">
@@ -1532,7 +1537,7 @@
       </c>
     </row>
     <row r="119" ht="15.75" customHeight="1">
-      <c r="A119" s="2">
+      <c r="A119" s="3">
         <v>41913</v>
       </c>
       <c r="B119" s="1">
@@ -1540,7 +1545,7 @@
       </c>
     </row>
     <row r="120" ht="15.75" customHeight="1">
-      <c r="A120" s="2">
+      <c r="A120" s="3">
         <v>41944</v>
       </c>
       <c r="B120" s="1">
@@ -1548,7 +1553,7 @@
       </c>
     </row>
     <row r="121" ht="15.75" customHeight="1">
-      <c r="A121" s="2">
+      <c r="A121" s="3">
         <v>41974</v>
       </c>
       <c r="B121" s="1">
@@ -1556,7 +1561,7 @@
       </c>
     </row>
     <row r="122" ht="15.75" customHeight="1">
-      <c r="A122" s="2">
+      <c r="A122" s="3">
         <v>42005</v>
       </c>
       <c r="B122" s="1">
@@ -1564,7 +1569,7 @@
       </c>
     </row>
     <row r="123" ht="15.75" customHeight="1">
-      <c r="A123" s="2">
+      <c r="A123" s="3">
         <v>42036</v>
       </c>
       <c r="B123" s="1">
@@ -1572,7 +1577,7 @@
       </c>
     </row>
     <row r="124" ht="15.75" customHeight="1">
-      <c r="A124" s="2">
+      <c r="A124" s="3">
         <v>42064</v>
       </c>
       <c r="B124" s="1">
@@ -1580,7 +1585,7 @@
       </c>
     </row>
     <row r="125" ht="15.75" customHeight="1">
-      <c r="A125" s="2">
+      <c r="A125" s="3">
         <v>42095</v>
       </c>
       <c r="B125" s="1">
@@ -1588,7 +1593,7 @@
       </c>
     </row>
     <row r="126" ht="15.75" customHeight="1">
-      <c r="A126" s="2">
+      <c r="A126" s="3">
         <v>42125</v>
       </c>
       <c r="B126" s="1">
@@ -1596,7 +1601,7 @@
       </c>
     </row>
     <row r="127" ht="15.75" customHeight="1">
-      <c r="A127" s="2">
+      <c r="A127" s="3">
         <v>42156</v>
       </c>
       <c r="B127" s="1">
@@ -1604,7 +1609,7 @@
       </c>
     </row>
     <row r="128" ht="15.75" customHeight="1">
-      <c r="A128" s="2">
+      <c r="A128" s="3">
         <v>42186</v>
       </c>
       <c r="B128" s="1">
@@ -1612,7 +1617,7 @@
       </c>
     </row>
     <row r="129" ht="15.75" customHeight="1">
-      <c r="A129" s="2">
+      <c r="A129" s="3">
         <v>42217</v>
       </c>
       <c r="B129" s="1">
@@ -1620,7 +1625,7 @@
       </c>
     </row>
     <row r="130" ht="15.75" customHeight="1">
-      <c r="A130" s="2">
+      <c r="A130" s="3">
         <v>42248</v>
       </c>
       <c r="B130" s="1">
@@ -1628,7 +1633,7 @@
       </c>
     </row>
     <row r="131" ht="15.75" customHeight="1">
-      <c r="A131" s="2">
+      <c r="A131" s="3">
         <v>42278</v>
       </c>
       <c r="B131" s="1">
@@ -1636,7 +1641,7 @@
       </c>
     </row>
     <row r="132" ht="15.75" customHeight="1">
-      <c r="A132" s="2">
+      <c r="A132" s="3">
         <v>42309</v>
       </c>
       <c r="B132" s="1">
@@ -1644,7 +1649,7 @@
       </c>
     </row>
     <row r="133" ht="15.75" customHeight="1">
-      <c r="A133" s="2">
+      <c r="A133" s="3">
         <v>42339</v>
       </c>
       <c r="B133" s="1">
@@ -1652,7 +1657,7 @@
       </c>
     </row>
     <row r="134" ht="15.75" customHeight="1">
-      <c r="A134" s="2">
+      <c r="A134" s="3">
         <v>42370</v>
       </c>
       <c r="B134" s="1">
@@ -1660,7 +1665,7 @@
       </c>
     </row>
     <row r="135" ht="15.75" customHeight="1">
-      <c r="A135" s="2">
+      <c r="A135" s="3">
         <v>42401</v>
       </c>
       <c r="B135" s="1">
@@ -1668,7 +1673,7 @@
       </c>
     </row>
     <row r="136" ht="15.75" customHeight="1">
-      <c r="A136" s="2">
+      <c r="A136" s="3">
         <v>42430</v>
       </c>
       <c r="B136" s="1">
@@ -1676,7 +1681,7 @@
       </c>
     </row>
     <row r="137" ht="15.75" customHeight="1">
-      <c r="A137" s="2">
+      <c r="A137" s="3">
         <v>42461</v>
       </c>
       <c r="B137" s="1">
@@ -1684,7 +1689,7 @@
       </c>
     </row>
     <row r="138" ht="15.75" customHeight="1">
-      <c r="A138" s="2">
+      <c r="A138" s="3">
         <v>42491</v>
       </c>
       <c r="B138" s="1">
@@ -1692,7 +1697,7 @@
       </c>
     </row>
     <row r="139" ht="15.75" customHeight="1">
-      <c r="A139" s="2">
+      <c r="A139" s="3">
         <v>42522</v>
       </c>
       <c r="B139" s="1">
@@ -1700,7 +1705,7 @@
       </c>
     </row>
     <row r="140" ht="15.75" customHeight="1">
-      <c r="A140" s="2">
+      <c r="A140" s="3">
         <v>42552</v>
       </c>
       <c r="B140" s="1">
@@ -1708,7 +1713,7 @@
       </c>
     </row>
     <row r="141" ht="15.75" customHeight="1">
-      <c r="A141" s="2">
+      <c r="A141" s="3">
         <v>42583</v>
       </c>
       <c r="B141" s="1">
@@ -1716,7 +1721,7 @@
       </c>
     </row>
     <row r="142" ht="15.75" customHeight="1">
-      <c r="A142" s="2">
+      <c r="A142" s="3">
         <v>42614</v>
       </c>
       <c r="B142" s="1">
@@ -1724,7 +1729,7 @@
       </c>
     </row>
     <row r="143" ht="15.75" customHeight="1">
-      <c r="A143" s="2">
+      <c r="A143" s="3">
         <v>42644</v>
       </c>
       <c r="B143" s="1">
@@ -1732,7 +1737,7 @@
       </c>
     </row>
     <row r="144" ht="15.75" customHeight="1">
-      <c r="A144" s="2">
+      <c r="A144" s="3">
         <v>42675</v>
       </c>
       <c r="B144" s="1">
@@ -1740,7 +1745,7 @@
       </c>
     </row>
     <row r="145" ht="15.75" customHeight="1">
-      <c r="A145" s="2">
+      <c r="A145" s="3">
         <v>42705</v>
       </c>
       <c r="B145" s="1">
@@ -1748,7 +1753,7 @@
       </c>
     </row>
     <row r="146" ht="15.75" customHeight="1">
-      <c r="A146" s="2">
+      <c r="A146" s="3">
         <v>42736</v>
       </c>
       <c r="B146" s="1">
@@ -1756,7 +1761,7 @@
       </c>
     </row>
     <row r="147" ht="15.75" customHeight="1">
-      <c r="A147" s="2">
+      <c r="A147" s="3">
         <v>42767</v>
       </c>
       <c r="B147" s="1">
@@ -1764,7 +1769,7 @@
       </c>
     </row>
     <row r="148" ht="15.75" customHeight="1">
-      <c r="A148" s="2">
+      <c r="A148" s="3">
         <v>42795</v>
       </c>
       <c r="B148" s="1">
@@ -1772,7 +1777,7 @@
       </c>
     </row>
     <row r="149" ht="15.75" customHeight="1">
-      <c r="A149" s="2">
+      <c r="A149" s="3">
         <v>42826</v>
       </c>
       <c r="B149" s="1">
@@ -1780,7 +1785,7 @@
       </c>
     </row>
     <row r="150" ht="15.75" customHeight="1">
-      <c r="A150" s="2">
+      <c r="A150" s="3">
         <v>42856</v>
       </c>
       <c r="B150" s="1">
@@ -1788,7 +1793,7 @@
       </c>
     </row>
     <row r="151" ht="15.75" customHeight="1">
-      <c r="A151" s="2">
+      <c r="A151" s="3">
         <v>42887</v>
       </c>
       <c r="B151" s="1">
@@ -1796,7 +1801,7 @@
       </c>
     </row>
     <row r="152" ht="15.75" customHeight="1">
-      <c r="A152" s="2">
+      <c r="A152" s="3">
         <v>42917</v>
       </c>
       <c r="B152" s="1">
@@ -1804,7 +1809,7 @@
       </c>
     </row>
     <row r="153" ht="15.75" customHeight="1">
-      <c r="A153" s="2">
+      <c r="A153" s="3">
         <v>42948</v>
       </c>
       <c r="B153" s="1">
@@ -1812,7 +1817,7 @@
       </c>
     </row>
     <row r="154" ht="15.75" customHeight="1">
-      <c r="A154" s="2">
+      <c r="A154" s="3">
         <v>42979</v>
       </c>
       <c r="B154" s="1">
@@ -1820,7 +1825,7 @@
       </c>
     </row>
     <row r="155" ht="15.75" customHeight="1">
-      <c r="A155" s="2">
+      <c r="A155" s="3">
         <v>43009</v>
       </c>
       <c r="B155" s="1">
@@ -1828,7 +1833,7 @@
       </c>
     </row>
     <row r="156" ht="15.75" customHeight="1">
-      <c r="A156" s="2">
+      <c r="A156" s="3">
         <v>43040</v>
       </c>
       <c r="B156" s="1">
@@ -1836,7 +1841,7 @@
       </c>
     </row>
     <row r="157" ht="15.75" customHeight="1">
-      <c r="A157" s="2">
+      <c r="A157" s="3">
         <v>43070</v>
       </c>
       <c r="B157" s="1">
@@ -1844,7 +1849,7 @@
       </c>
     </row>
     <row r="158" ht="15.75" customHeight="1">
-      <c r="A158" s="2">
+      <c r="A158" s="3">
         <v>43101</v>
       </c>
       <c r="B158" s="1">
@@ -1852,7 +1857,7 @@
       </c>
     </row>
     <row r="159" ht="15.75" customHeight="1">
-      <c r="A159" s="2">
+      <c r="A159" s="3">
         <v>43132</v>
       </c>
       <c r="B159" s="1">
@@ -1860,7 +1865,7 @@
       </c>
     </row>
     <row r="160" ht="15.75" customHeight="1">
-      <c r="A160" s="2">
+      <c r="A160" s="3">
         <v>43160</v>
       </c>
       <c r="B160" s="1">
@@ -1868,7 +1873,7 @@
       </c>
     </row>
     <row r="161" ht="15.75" customHeight="1">
-      <c r="A161" s="2">
+      <c r="A161" s="3">
         <v>43191</v>
       </c>
       <c r="B161" s="1">
@@ -1876,7 +1881,7 @@
       </c>
     </row>
     <row r="162" ht="15.75" customHeight="1">
-      <c r="A162" s="2">
+      <c r="A162" s="3">
         <v>43221</v>
       </c>
       <c r="B162" s="1">
@@ -1884,7 +1889,7 @@
       </c>
     </row>
     <row r="163" ht="15.75" customHeight="1">
-      <c r="A163" s="2">
+      <c r="A163" s="3">
         <v>43252</v>
       </c>
       <c r="B163" s="1">
@@ -1892,7 +1897,7 @@
       </c>
     </row>
     <row r="164" ht="15.75" customHeight="1">
-      <c r="A164" s="2">
+      <c r="A164" s="3">
         <v>43282</v>
       </c>
       <c r="B164" s="1">
@@ -1900,7 +1905,7 @@
       </c>
     </row>
     <row r="165" ht="15.75" customHeight="1">
-      <c r="A165" s="2">
+      <c r="A165" s="3">
         <v>43313</v>
       </c>
       <c r="B165" s="1">
@@ -1908,7 +1913,7 @@
       </c>
     </row>
     <row r="166" ht="15.75" customHeight="1">
-      <c r="A166" s="2">
+      <c r="A166" s="3">
         <v>43344</v>
       </c>
       <c r="B166" s="1">
@@ -1916,7 +1921,7 @@
       </c>
     </row>
     <row r="167" ht="15.75" customHeight="1">
-      <c r="A167" s="2">
+      <c r="A167" s="3">
         <v>43374</v>
       </c>
       <c r="B167" s="1">
@@ -1924,7 +1929,7 @@
       </c>
     </row>
     <row r="168" ht="15.75" customHeight="1">
-      <c r="A168" s="2">
+      <c r="A168" s="3">
         <v>43405</v>
       </c>
       <c r="B168" s="1">
@@ -1932,7 +1937,7 @@
       </c>
     </row>
     <row r="169" ht="15.75" customHeight="1">
-      <c r="A169" s="2">
+      <c r="A169" s="3">
         <v>43435</v>
       </c>
       <c r="B169" s="1">
@@ -1940,7 +1945,7 @@
       </c>
     </row>
     <row r="170" ht="15.75" customHeight="1">
-      <c r="A170" s="2">
+      <c r="A170" s="3">
         <v>43466</v>
       </c>
       <c r="B170" s="1">
@@ -1948,7 +1953,7 @@
       </c>
     </row>
     <row r="171" ht="15.75" customHeight="1">
-      <c r="A171" s="2">
+      <c r="A171" s="3">
         <v>43497</v>
       </c>
       <c r="B171" s="1">
@@ -1956,7 +1961,7 @@
       </c>
     </row>
     <row r="172" ht="15.75" customHeight="1">
-      <c r="A172" s="2">
+      <c r="A172" s="3">
         <v>43525</v>
       </c>
       <c r="B172" s="1">
@@ -1964,7 +1969,7 @@
       </c>
     </row>
     <row r="173" ht="15.75" customHeight="1">
-      <c r="A173" s="2">
+      <c r="A173" s="3">
         <v>43556</v>
       </c>
       <c r="B173" s="1">
@@ -1972,7 +1977,7 @@
       </c>
     </row>
     <row r="174" ht="15.75" customHeight="1">
-      <c r="A174" s="2">
+      <c r="A174" s="3">
         <v>43586</v>
       </c>
       <c r="B174" s="1">
@@ -1980,7 +1985,7 @@
       </c>
     </row>
     <row r="175" ht="15.75" customHeight="1">
-      <c r="A175" s="2">
+      <c r="A175" s="3">
         <v>43617</v>
       </c>
       <c r="B175" s="1">
@@ -1988,7 +1993,7 @@
       </c>
     </row>
     <row r="176" ht="15.75" customHeight="1">
-      <c r="A176" s="2">
+      <c r="A176" s="3">
         <v>43647</v>
       </c>
       <c r="B176" s="1">
@@ -1996,7 +2001,7 @@
       </c>
     </row>
     <row r="177" ht="15.75" customHeight="1">
-      <c r="A177" s="2">
+      <c r="A177" s="3">
         <v>43678</v>
       </c>
       <c r="B177" s="1">
@@ -2004,7 +2009,7 @@
       </c>
     </row>
     <row r="178" ht="15.75" customHeight="1">
-      <c r="A178" s="2">
+      <c r="A178" s="3">
         <v>43709</v>
       </c>
       <c r="B178" s="1">
@@ -2012,7 +2017,7 @@
       </c>
     </row>
     <row r="179" ht="15.75" customHeight="1">
-      <c r="A179" s="2">
+      <c r="A179" s="3">
         <v>43739</v>
       </c>
       <c r="B179" s="1">
@@ -2020,7 +2025,7 @@
       </c>
     </row>
     <row r="180" ht="15.75" customHeight="1">
-      <c r="A180" s="2">
+      <c r="A180" s="3">
         <v>43770</v>
       </c>
       <c r="B180" s="1">
@@ -2028,7 +2033,7 @@
       </c>
     </row>
     <row r="181" ht="15.75" customHeight="1">
-      <c r="A181" s="2">
+      <c r="A181" s="3">
         <v>43800</v>
       </c>
       <c r="B181" s="1">
@@ -2036,7 +2041,7 @@
       </c>
     </row>
     <row r="182" ht="15.75" customHeight="1">
-      <c r="A182" s="2">
+      <c r="A182" s="3">
         <v>43831</v>
       </c>
       <c r="B182" s="1">
@@ -2044,7 +2049,7 @@
       </c>
     </row>
     <row r="183" ht="15.75" customHeight="1">
-      <c r="A183" s="2">
+      <c r="A183" s="3">
         <v>43862</v>
       </c>
       <c r="B183" s="1">
@@ -2052,7 +2057,7 @@
       </c>
     </row>
     <row r="184" ht="15.75" customHeight="1">
-      <c r="A184" s="2">
+      <c r="A184" s="3">
         <v>43891</v>
       </c>
       <c r="B184" s="1">
@@ -2060,7 +2065,7 @@
       </c>
     </row>
     <row r="185" ht="15.75" customHeight="1">
-      <c r="A185" s="2">
+      <c r="A185" s="3">
         <v>43922</v>
       </c>
       <c r="B185" s="1">
@@ -2068,7 +2073,7 @@
       </c>
     </row>
     <row r="186" ht="15.75" customHeight="1">
-      <c r="A186" s="2">
+      <c r="A186" s="3">
         <v>43952</v>
       </c>
       <c r="B186" s="1">
@@ -2076,7 +2081,7 @@
       </c>
     </row>
     <row r="187" ht="15.75" customHeight="1">
-      <c r="A187" s="2">
+      <c r="A187" s="3">
         <v>43983</v>
       </c>
       <c r="B187" s="1">
@@ -2084,7 +2089,7 @@
       </c>
     </row>
     <row r="188" ht="15.75" customHeight="1">
-      <c r="A188" s="2">
+      <c r="A188" s="3">
         <v>44013</v>
       </c>
       <c r="B188" s="1">
@@ -2092,7 +2097,7 @@
       </c>
     </row>
     <row r="189" ht="15.75" customHeight="1">
-      <c r="A189" s="2">
+      <c r="A189" s="3">
         <v>44044</v>
       </c>
       <c r="B189" s="1">
@@ -2100,7 +2105,7 @@
       </c>
     </row>
     <row r="190" ht="15.75" customHeight="1">
-      <c r="A190" s="2">
+      <c r="A190" s="3">
         <v>44075</v>
       </c>
       <c r="B190" s="1">
@@ -2108,7 +2113,7 @@
       </c>
     </row>
     <row r="191" ht="15.75" customHeight="1">
-      <c r="A191" s="2">
+      <c r="A191" s="3">
         <v>44105</v>
       </c>
       <c r="B191" s="1">
@@ -2116,7 +2121,7 @@
       </c>
     </row>
     <row r="192" ht="15.75" customHeight="1">
-      <c r="A192" s="2">
+      <c r="A192" s="3">
         <v>44136</v>
       </c>
       <c r="B192" s="1">
@@ -2124,7 +2129,7 @@
       </c>
     </row>
     <row r="193" ht="15.75" customHeight="1">
-      <c r="A193" s="2">
+      <c r="A193" s="3">
         <v>44166</v>
       </c>
       <c r="B193" s="1">
@@ -2132,7 +2137,7 @@
       </c>
     </row>
     <row r="194" ht="15.75" customHeight="1">
-      <c r="A194" s="2">
+      <c r="A194" s="3">
         <v>44197</v>
       </c>
       <c r="B194" s="1">
@@ -2140,7 +2145,7 @@
       </c>
     </row>
     <row r="195" ht="15.75" customHeight="1">
-      <c r="A195" s="2">
+      <c r="A195" s="3">
         <v>44228</v>
       </c>
       <c r="B195" s="1">
@@ -2148,7 +2153,7 @@
       </c>
     </row>
     <row r="196" ht="15.75" customHeight="1">
-      <c r="A196" s="2">
+      <c r="A196" s="3">
         <v>44256</v>
       </c>
       <c r="B196" s="1">
@@ -2156,7 +2161,7 @@
       </c>
     </row>
     <row r="197" ht="15.75" customHeight="1">
-      <c r="A197" s="2">
+      <c r="A197" s="3">
         <v>44287</v>
       </c>
       <c r="B197" s="1">
@@ -2164,7 +2169,7 @@
       </c>
     </row>
     <row r="198" ht="15.75" customHeight="1">
-      <c r="A198" s="2">
+      <c r="A198" s="3">
         <v>44317</v>
       </c>
       <c r="B198" s="1">
@@ -2172,7 +2177,7 @@
       </c>
     </row>
     <row r="199" ht="15.75" customHeight="1">
-      <c r="A199" s="2">
+      <c r="A199" s="3">
         <v>44348</v>
       </c>
       <c r="B199" s="1">
@@ -2180,7 +2185,7 @@
       </c>
     </row>
     <row r="200" ht="15.75" customHeight="1">
-      <c r="A200" s="2">
+      <c r="A200" s="3">
         <v>44378</v>
       </c>
       <c r="B200" s="1">
@@ -2188,7 +2193,7 @@
       </c>
     </row>
     <row r="201" ht="15.75" customHeight="1">
-      <c r="A201" s="2">
+      <c r="A201" s="3">
         <v>44409</v>
       </c>
       <c r="B201" s="1">
@@ -2196,7 +2201,7 @@
       </c>
     </row>
     <row r="202" ht="15.75" customHeight="1">
-      <c r="A202" s="2">
+      <c r="A202" s="3">
         <v>44440</v>
       </c>
       <c r="B202" s="1">
@@ -2204,7 +2209,7 @@
       </c>
     </row>
     <row r="203" ht="15.75" customHeight="1">
-      <c r="A203" s="2">
+      <c r="A203" s="3">
         <v>44470</v>
       </c>
       <c r="B203" s="1">
@@ -2212,7 +2217,7 @@
       </c>
     </row>
     <row r="204" ht="15.75" customHeight="1">
-      <c r="A204" s="2">
+      <c r="A204" s="3">
         <v>44501</v>
       </c>
       <c r="B204" s="1">
@@ -2220,7 +2225,7 @@
       </c>
     </row>
     <row r="205" ht="15.75" customHeight="1">
-      <c r="A205" s="2">
+      <c r="A205" s="3">
         <v>44531</v>
       </c>
       <c r="B205" s="1">
@@ -2228,7 +2233,7 @@
       </c>
     </row>
     <row r="206" ht="15.75" customHeight="1">
-      <c r="A206" s="2">
+      <c r="A206" s="3">
         <v>44562</v>
       </c>
       <c r="B206" s="1">
@@ -2236,7 +2241,7 @@
       </c>
     </row>
     <row r="207" ht="15.75" customHeight="1">
-      <c r="A207" s="2">
+      <c r="A207" s="3">
         <v>44593</v>
       </c>
       <c r="B207" s="1">
@@ -2244,7 +2249,7 @@
       </c>
     </row>
     <row r="208" ht="15.75" customHeight="1">
-      <c r="A208" s="2">
+      <c r="A208" s="3">
         <v>44621</v>
       </c>
       <c r="B208" s="1">
@@ -2252,7 +2257,7 @@
       </c>
     </row>
     <row r="209" ht="15.75" customHeight="1">
-      <c r="A209" s="2">
+      <c r="A209" s="3">
         <v>44652</v>
       </c>
       <c r="B209" s="1">
@@ -2260,7 +2265,7 @@
       </c>
     </row>
     <row r="210" ht="15.75" customHeight="1">
-      <c r="A210" s="2">
+      <c r="A210" s="3">
         <v>44682</v>
       </c>
       <c r="B210" s="1">
@@ -2268,7 +2273,7 @@
       </c>
     </row>
     <row r="211" ht="15.75" customHeight="1">
-      <c r="A211" s="2">
+      <c r="A211" s="3">
         <v>44713</v>
       </c>
       <c r="B211" s="1">
@@ -2276,7 +2281,7 @@
       </c>
     </row>
     <row r="212" ht="15.75" customHeight="1">
-      <c r="A212" s="2">
+      <c r="A212" s="3">
         <v>44743</v>
       </c>
       <c r="B212" s="1">
@@ -2284,7 +2289,7 @@
       </c>
     </row>
     <row r="213" ht="15.75" customHeight="1">
-      <c r="A213" s="2">
+      <c r="A213" s="3">
         <v>44774</v>
       </c>
       <c r="B213" s="1">
@@ -2292,7 +2297,7 @@
       </c>
     </row>
     <row r="214" ht="15.75" customHeight="1">
-      <c r="A214" s="2">
+      <c r="A214" s="3">
         <v>44805</v>
       </c>
       <c r="B214" s="1">
@@ -2300,7 +2305,7 @@
       </c>
     </row>
     <row r="215" ht="15.75" customHeight="1">
-      <c r="A215" s="2">
+      <c r="A215" s="3">
         <v>44835</v>
       </c>
       <c r="B215" s="1">
@@ -2308,7 +2313,7 @@
       </c>
     </row>
     <row r="216" ht="15.75" customHeight="1">
-      <c r="A216" s="2">
+      <c r="A216" s="3">
         <v>44866</v>
       </c>
       <c r="B216" s="1">
@@ -2316,7 +2321,7 @@
       </c>
     </row>
     <row r="217" ht="15.75" customHeight="1">
-      <c r="A217" s="2">
+      <c r="A217" s="3">
         <v>44896</v>
       </c>
       <c r="B217" s="1">
@@ -2324,7 +2329,7 @@
       </c>
     </row>
     <row r="218" ht="15.75" customHeight="1">
-      <c r="A218" s="2">
+      <c r="A218" s="3">
         <v>44927</v>
       </c>
       <c r="B218" s="1">
@@ -2332,7 +2337,7 @@
       </c>
     </row>
     <row r="219" ht="15.75" customHeight="1">
-      <c r="A219" s="2">
+      <c r="A219" s="3">
         <v>44958</v>
       </c>
       <c r="B219" s="1">
@@ -2340,7 +2345,7 @@
       </c>
     </row>
     <row r="220" ht="15.75" customHeight="1">
-      <c r="A220" s="2">
+      <c r="A220" s="3">
         <v>44986</v>
       </c>
       <c r="B220" s="1">
@@ -2348,7 +2353,7 @@
       </c>
     </row>
     <row r="221" ht="15.75" customHeight="1">
-      <c r="A221" s="2">
+      <c r="A221" s="3">
         <v>45017</v>
       </c>
       <c r="B221" s="1">
@@ -2356,7 +2361,7 @@
       </c>
     </row>
     <row r="222" ht="15.75" customHeight="1">
-      <c r="A222" s="2">
+      <c r="A222" s="3">
         <v>45047</v>
       </c>
       <c r="B222" s="1">
@@ -2364,7 +2369,7 @@
       </c>
     </row>
     <row r="223" ht="15.75" customHeight="1">
-      <c r="A223" s="2">
+      <c r="A223" s="3">
         <v>45078</v>
       </c>
       <c r="B223" s="1">
@@ -2372,7 +2377,7 @@
       </c>
     </row>
     <row r="224" ht="15.75" customHeight="1">
-      <c r="A224" s="2">
+      <c r="A224" s="3">
         <v>45108</v>
       </c>
       <c r="B224" s="1">
@@ -2380,7 +2385,7 @@
       </c>
     </row>
     <row r="225" ht="15.75" customHeight="1">
-      <c r="A225" s="2">
+      <c r="A225" s="3">
         <v>45139</v>
       </c>
       <c r="B225" s="1">
@@ -2388,7 +2393,7 @@
       </c>
     </row>
     <row r="226" ht="15.75" customHeight="1">
-      <c r="A226" s="2">
+      <c r="A226" s="3">
         <v>45170</v>
       </c>
       <c r="B226" s="1">
@@ -2396,7 +2401,7 @@
       </c>
     </row>
     <row r="227" ht="15.75" customHeight="1">
-      <c r="A227" s="2">
+      <c r="A227" s="3">
         <v>45200</v>
       </c>
       <c r="B227" s="1">
@@ -2404,7 +2409,7 @@
       </c>
     </row>
     <row r="228" ht="15.75" customHeight="1">
-      <c r="A228" s="2">
+      <c r="A228" s="3">
         <v>45231</v>
       </c>
       <c r="B228" s="1">
@@ -2412,7 +2417,7 @@
       </c>
     </row>
     <row r="229" ht="15.75" customHeight="1">
-      <c r="A229" s="2">
+      <c r="A229" s="3">
         <v>45261</v>
       </c>
       <c r="B229" s="1">
@@ -2420,7 +2425,7 @@
       </c>
     </row>
     <row r="230" ht="15.75" customHeight="1">
-      <c r="A230" s="2">
+      <c r="A230" s="3">
         <v>45292</v>
       </c>
       <c r="B230" s="1">
@@ -2428,7 +2433,7 @@
       </c>
     </row>
     <row r="231" ht="15.75" customHeight="1">
-      <c r="A231" s="2">
+      <c r="A231" s="3">
         <v>45323</v>
       </c>
       <c r="B231" s="1">
@@ -2436,7 +2441,7 @@
       </c>
     </row>
     <row r="232" ht="15.75" customHeight="1">
-      <c r="A232" s="2">
+      <c r="A232" s="3">
         <v>45352</v>
       </c>
       <c r="B232" s="1">
@@ -2444,7 +2449,7 @@
       </c>
     </row>
     <row r="233" ht="15.75" customHeight="1">
-      <c r="A233" s="2">
+      <c r="A233" s="3">
         <v>45383</v>
       </c>
       <c r="B233" s="1">
@@ -2452,7 +2457,7 @@
       </c>
     </row>
     <row r="234" ht="15.75" customHeight="1">
-      <c r="A234" s="2">
+      <c r="A234" s="3">
         <v>45413</v>
       </c>
       <c r="B234" s="1">
@@ -2460,7 +2465,7 @@
       </c>
     </row>
     <row r="235" ht="15.75" customHeight="1">
-      <c r="A235" s="2">
+      <c r="A235" s="3">
         <v>45444</v>
       </c>
       <c r="B235" s="1">
@@ -2468,7 +2473,7 @@
       </c>
     </row>
     <row r="236" ht="15.75" customHeight="1">
-      <c r="A236" s="2">
+      <c r="A236" s="3">
         <v>45474</v>
       </c>
       <c r="B236" s="1">
@@ -2476,7 +2481,7 @@
       </c>
     </row>
     <row r="237" ht="15.75" customHeight="1">
-      <c r="A237" s="2">
+      <c r="A237" s="3">
         <v>45505</v>
       </c>
       <c r="B237" s="1">
@@ -2484,7 +2489,7 @@
       </c>
     </row>
     <row r="238" ht="15.75" customHeight="1">
-      <c r="A238" s="2">
+      <c r="A238" s="3">
         <v>45536</v>
       </c>
       <c r="B238" s="1">
@@ -2492,7 +2497,7 @@
       </c>
     </row>
     <row r="239" ht="15.75" customHeight="1">
-      <c r="A239" s="2">
+      <c r="A239" s="3">
         <v>45566</v>
       </c>
       <c r="B239" s="1">
@@ -2500,7 +2505,7 @@
       </c>
     </row>
     <row r="240" ht="15.75" customHeight="1">
-      <c r="A240" s="2">
+      <c r="A240" s="3">
         <v>45597</v>
       </c>
       <c r="B240" s="1">
@@ -2508,7 +2513,7 @@
       </c>
     </row>
     <row r="241" ht="15.75" customHeight="1">
-      <c r="A241" s="2">
+      <c r="A241" s="3">
         <v>45627</v>
       </c>
       <c r="B241" s="1">
@@ -2516,7 +2521,7 @@
       </c>
     </row>
     <row r="242" ht="15.75" customHeight="1">
-      <c r="A242" s="2">
+      <c r="A242" s="3">
         <v>45658</v>
       </c>
       <c r="B242" s="1">
@@ -2524,16 +2529,16 @@
       </c>
     </row>
     <row r="243" ht="15.75" customHeight="1">
-      <c r="A243" s="2">
+      <c r="A243" s="3">
         <v>45689</v>
       </c>
       <c r="B243" s="1">
         <v>599.24000000000001</v>
       </c>
-      <c r="H243" s="3"/>
+      <c r="H243" s="4"/>
     </row>
     <row r="244" ht="15.75" customHeight="1">
-      <c r="A244" s="2">
+      <c r="A244" s="3">
         <v>45717</v>
       </c>
       <c r="B244" s="1">
@@ -2541,7 +2546,7 @@
       </c>
     </row>
     <row r="245" ht="15.75" customHeight="1">
-      <c r="A245" s="2">
+      <c r="A245" s="3">
         <v>45748</v>
       </c>
       <c r="B245" s="1">
@@ -2549,15 +2554,15 @@
       </c>
     </row>
     <row r="246" ht="15.75" customHeight="1">
-      <c r="A246" s="2">
+      <c r="A246" s="3">
         <v>45778</v>
       </c>
-      <c r="B246">
+      <c r="B246" s="1">
         <v>588.08000000000004</v>
       </c>
     </row>
     <row r="247" ht="15.75" customHeight="1">
-      <c r="A247" s="2">
+      <c r="A247" s="3">
         <v>45809</v>
       </c>
       <c r="B247" s="1">
@@ -2565,7 +2570,7 @@
       </c>
     </row>
     <row r="248" ht="15.75" customHeight="1">
-      <c r="A248" s="2">
+      <c r="A248" s="3">
         <v>45839</v>
       </c>
       <c r="B248" s="1">
@@ -2573,7 +2578,7 @@
       </c>
     </row>
     <row r="249" ht="15.75" customHeight="1">
-      <c r="A249" s="2">
+      <c r="A249" s="3">
         <v>45870</v>
       </c>
       <c r="B249" s="1">
@@ -2581,7 +2586,7 @@
       </c>
     </row>
     <row r="250" ht="15.75" customHeight="1">
-      <c r="A250" s="2">
+      <c r="A250" s="3">
         <v>45901</v>
       </c>
       <c r="B250" s="1">
@@ -2589,7 +2594,7 @@
       </c>
     </row>
     <row r="251" ht="15.75" customHeight="1">
-      <c r="A251" s="2">
+      <c r="A251" s="3">
         <v>45931</v>
       </c>
       <c r="B251" s="1">
@@ -2597,7 +2602,7 @@
       </c>
     </row>
     <row r="252" ht="15.75" customHeight="1">
-      <c r="A252" s="2">
+      <c r="A252" s="3">
         <v>45962</v>
       </c>
       <c r="B252" s="1">
@@ -2605,38 +2610,45 @@
       </c>
     </row>
     <row r="253" ht="15.75" customHeight="1">
-      <c r="A253" s="4">
+      <c r="A253" s="5">
         <v>45992</v>
       </c>
-      <c r="B253">
+      <c r="B253" s="1">
         <v>572.74000000000001</v>
       </c>
     </row>
     <row r="254" ht="15.75" customHeight="1">
-      <c r="A254" s="4">
+      <c r="A254" s="5">
         <v>46023</v>
       </c>
-      <c r="B254">
+      <c r="B254" s="1">
         <v>577.25</v>
       </c>
     </row>
     <row r="255" ht="15.75" customHeight="1">
-      <c r="A255" s="4">
+      <c r="A255" s="5">
         <v>46054</v>
       </c>
-      <c r="B255">
+      <c r="B255" s="1">
         <v>579.51999999999998</v>
       </c>
     </row>
     <row r="256" ht="15.75" customHeight="1">
-      <c r="A256" s="4">
+      <c r="A256" s="5">
         <v>46082</v>
       </c>
-      <c r="B256">
+      <c r="B256" s="1">
         <v>612.80999999999995</v>
       </c>
     </row>
-    <row r="257" ht="15.75" customHeight="1"/>
+    <row r="257" ht="15.75" customHeight="1">
+      <c r="A257" s="3">
+        <v>46026</v>
+      </c>
+      <c r="B257" s="1">
+        <v>648.57000000000005</v>
+      </c>
+    </row>
     <row r="258" ht="15.75" customHeight="1"/>
     <row r="259" ht="15.75" customHeight="1"/>
     <row r="260" ht="15.75" customHeight="1"/>

</xml_diff>